<commit_message>
Exclude SuSy PYA rows; find header and PHI columns by name
- SuSy: header via "Disbursement Number", stop at PYA section, skip rows without a disbursement number
- PHI columns between programme/amount column and TOTAL (GBP and SuSy)
- PHI mapping for all clusters; ignore *.ipynb

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02 SuSy Disbursement File/Monthly Mar26 and FY25Q4 Subvention Disbursement Spreadsheet - NHG Mock.xlsx
+++ b/02 SuSy Disbursement File/Monthly Mar26 and FY25Q4 Subvention Disbursement Spreadsheet - NHG Mock.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limqi\Desktop\Subvention\SuSy Disbursement File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limqi\Desktop\Subvention\02 SuSy Disbursement File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0474D5-08E9-49F5-9A56-05D168FDAAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548F8845-C2FA-4FC1-B3A2-38E512A57175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="162">
   <si>
     <t>Budget as at 01_03_2026 - For 3_2026</t>
   </si>
@@ -488,6 +488,24 @@
   </si>
   <si>
     <t>Miscellaneous Funding Adjustments</t>
+  </si>
+  <si>
+    <t>3.29</t>
+  </si>
+  <si>
+    <t>Prior Years' Adjustments (PYAs):</t>
+  </si>
+  <si>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>D000005040</t>
+  </si>
+  <si>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>D000005041</t>
   </si>
 </sst>
 </file>
@@ -554,7 +572,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -562,6 +580,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -876,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB52"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3034,7 +3053,187 @@
         <v>51566204</v>
       </c>
     </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>38</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D48" t="s">
+        <v>127</v>
+      </c>
+      <c r="F48" s="1">
+        <v>12345678</v>
+      </c>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1">
+        <v>12345678</v>
+      </c>
+      <c r="I48" s="1"/>
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1"/>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="1"/>
+      <c r="R48" s="1"/>
+      <c r="S48" s="1"/>
+      <c r="T48" s="1"/>
+      <c r="U48" s="1"/>
+      <c r="V48" s="1"/>
+      <c r="W48" s="1"/>
+      <c r="X48" s="1"/>
+      <c r="Y48" s="1"/>
+      <c r="Z48" s="1"/>
+      <c r="AA48" s="1"/>
+      <c r="AB48" s="1">
+        <v>12345678</v>
+      </c>
+    </row>
+    <row r="49" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+      <c r="J49" s="1"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1"/>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
+      <c r="S49" s="1"/>
+      <c r="T49" s="1"/>
+      <c r="U49" s="1"/>
+      <c r="V49" s="1"/>
+      <c r="W49" s="1"/>
+      <c r="X49" s="1"/>
+      <c r="Y49" s="1"/>
+      <c r="Z49" s="1"/>
+      <c r="AA49" s="1"/>
+      <c r="AB49" s="1"/>
+    </row>
+    <row r="50" spans="1:28" ht="13.15" x14ac:dyDescent="0.4">
+      <c r="D50" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
+      <c r="S50" s="1"/>
+      <c r="T50" s="1"/>
+      <c r="U50" s="1"/>
+      <c r="V50" s="1"/>
+      <c r="W50" s="1"/>
+      <c r="X50" s="1"/>
+      <c r="Y50" s="1"/>
+      <c r="Z50" s="1"/>
+      <c r="AA50" s="1"/>
+      <c r="AB50" s="1"/>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>33</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C51" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51" t="s">
+        <v>127</v>
+      </c>
+      <c r="F51" s="1">
+        <v>5555555</v>
+      </c>
+      <c r="G51" s="1">
+        <v>5555555</v>
+      </c>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
+      <c r="J51" s="1"/>
+      <c r="K51" s="1"/>
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+      <c r="N51" s="1"/>
+      <c r="O51" s="1"/>
+      <c r="P51" s="1"/>
+      <c r="Q51" s="1"/>
+      <c r="R51" s="1"/>
+      <c r="S51" s="1"/>
+      <c r="T51" s="1"/>
+      <c r="U51" s="1"/>
+      <c r="V51" s="1"/>
+      <c r="W51" s="1"/>
+      <c r="X51" s="1"/>
+      <c r="Y51" s="1"/>
+      <c r="Z51" s="1"/>
+      <c r="AA51" s="1"/>
+      <c r="AB51" s="1">
+        <v>5555555</v>
+      </c>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>33</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C52" t="s">
+        <v>161</v>
+      </c>
+      <c r="D52" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" s="1">
+        <v>4444444</v>
+      </c>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1">
+        <v>4444444</v>
+      </c>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
+      <c r="T52" s="1"/>
+      <c r="U52" s="1"/>
+      <c r="V52" s="1"/>
+      <c r="W52" s="1"/>
+      <c r="X52" s="1"/>
+      <c r="Y52" s="1"/>
+      <c r="Z52" s="1"/>
+      <c r="AA52" s="1"/>
+      <c r="AB52" s="1">
+        <v>4444444</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>